<commit_message>
aumento de pruebas para la API
</commit_message>
<xml_diff>
--- a/Matriz de pruebas.xlsx
+++ b/Matriz de pruebas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Legion\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Legion\API_DGIDA_LOCAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F576F14E-3BEF-4BE2-820A-444D85FB5226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F541E3D-6686-49A9-8AAD-D3E4B971D08D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EC80005D-8709-4946-A325-33F6775FDC6E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="77">
   <si>
     <t>METODO</t>
   </si>
@@ -320,6 +320,15 @@
   </si>
   <si>
     <t>id_programa=PRG-cca3777c</t>
+  </si>
+  <si>
+    <t>{
+  "nombre": "Autoridad Agua",
+  "departamento_sede": "Sonsonate",
+  "municipio_sede": "Nahuizalco",
+  "telefono": "2612-3927",
+  "correo": "info.autoridad.agua@gob.sv"
+}</t>
   </si>
 </sst>
 </file>
@@ -742,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE5D9706-59AF-4BFA-9458-4FEEBE1C81DF}">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -1159,6 +1168,34 @@
         <v>18</v>
       </c>
     </row>
+    <row r="17" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" s="6"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
@@ -1175,9 +1212,10 @@
     <hyperlink ref="D14" r:id="rId11" xr:uid="{A9A0F352-1BA6-472A-8224-45F7C12ECFC4}"/>
     <hyperlink ref="D15" r:id="rId12" xr:uid="{1AF9EF42-996C-4D42-9FA0-3446A12AAC1A}"/>
     <hyperlink ref="D12" r:id="rId13" xr:uid="{1E6D8DDF-F050-4BAD-A43F-EFFD6D236299}"/>
+    <hyperlink ref="D17" r:id="rId14" xr:uid="{402A6020-52CD-467A-BDC7-E4E94831C403}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId14"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
 

</xml_diff>